<commit_message>
highlighted changes made with comments, adjusted spec files to include raw table/field names (with whitespaced removed) and cleaned up names (under snake columns), clean up table/field names post spec-comparison
</commit_message>
<xml_diff>
--- a/data-raw/techdatareport-tables.xlsx
+++ b/data-raw/techdatareport-tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://technomics.sharepoint.us/Projects/DOD/Army/TACOM/Stryker/Task 0003 - Stryker CSDR and Contracts CY21-25/Technical/TDR M&amp;R Dev/Read Files/TDR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bellenbogen\Software\R\readflexfile\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="14_{5267C218-CF8F-41F8-BFAC-ED3B2E4EDAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F537873B-FE2F-4AFC-B516-7CFD45E6F7BE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A0E1DC-F298-4B15-85F6-3BE87C092BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10560" yWindow="2175" windowWidth="12045" windowHeight="12090" activeTab="1" xr2:uid="{B45BC891-6358-4EB6-8DF4-312547779ABA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B45BC891-6358-4EB6-8DF4-312547779ABA}"/>
   </bookViews>
   <sheets>
     <sheet name="tables" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="109">
   <si>
     <t>table</t>
   </si>
@@ -49,48 +49,30 @@
     <t>ReportMetadata</t>
   </si>
   <si>
-    <t>reportmetadata</t>
-  </si>
-  <si>
     <t>submission</t>
   </si>
   <si>
     <t>OrderOrLot</t>
   </si>
   <si>
-    <t>ordersorlots</t>
-  </si>
-  <si>
     <t>EndItems</t>
   </si>
   <si>
     <t>EndItem</t>
   </si>
   <si>
-    <t>enditems</t>
-  </si>
-  <si>
     <t>WBS</t>
   </si>
   <si>
     <t>WBSElement</t>
   </si>
   <si>
-    <t>wbs</t>
-  </si>
-  <si>
     <t>TechnicalDataParameters</t>
   </si>
   <si>
-    <t>technicaldataparameters</t>
-  </si>
-  <si>
     <t>WBSMapping</t>
   </si>
   <si>
-    <t>wbsmapping</t>
-  </si>
-  <si>
     <t>field</t>
   </si>
   <si>
@@ -115,27 +97,15 @@
     <t>SecurityClassification</t>
   </si>
   <si>
-    <t>security_classification</t>
-  </si>
-  <si>
     <t>VARCHAR</t>
   </si>
   <si>
     <t>ProprietaryStatement</t>
   </si>
   <si>
-    <t>proprietary_statement</t>
-  </si>
-  <si>
     <t>ProgramName</t>
   </si>
   <si>
-    <t>program_name</t>
-  </si>
-  <si>
-    <t>phase_or_milestone_id</t>
-  </si>
-  <si>
     <t>PhaseOrMilestoneEnum</t>
   </si>
   <si>
@@ -145,243 +115,96 @@
     <t>PrimeMissionProduct</t>
   </si>
   <si>
-    <t>prime_mission_product</t>
-  </si>
-  <si>
     <t>CommodityType</t>
   </si>
   <si>
-    <t>commodity_type</t>
-  </si>
-  <si>
-    <t>reporting_organization_organization_name</t>
-  </si>
-  <si>
-    <t>reporting_organization_division_name</t>
-  </si>
-  <si>
-    <t>reporting_organization_cage_code</t>
-  </si>
-  <si>
-    <t>reporting_organization_location_street</t>
-  </si>
-  <si>
-    <t>reporting_organization_location_city</t>
-  </si>
-  <si>
-    <t>reporting_organization_location_state</t>
-  </si>
-  <si>
-    <t>reporting_organization_location_zip_code</t>
-  </si>
-  <si>
-    <t>reporting_organization_location_country</t>
-  </si>
-  <si>
     <t>ApprovedPlanNumber</t>
   </si>
   <si>
-    <t>approved_plan_number</t>
-  </si>
-  <si>
     <t>ApprovedPlanRevisionNumber</t>
   </si>
   <si>
-    <t>approved_plan_revision_number</t>
-  </si>
-  <si>
     <t>CustomerName</t>
   </si>
   <si>
-    <t>customer_name</t>
-  </si>
-  <si>
     <t>ContractTypeID</t>
   </si>
   <si>
-    <t>contract_type_id</t>
-  </si>
-  <si>
     <t>ContractTypeEnum</t>
   </si>
   <si>
     <t>ContractPrice</t>
   </si>
   <si>
-    <t>contract_price</t>
-  </si>
-  <si>
     <t>DOUBLE</t>
   </si>
   <si>
     <t>ContractCeiling</t>
   </si>
   <si>
-    <t>contract_ceiling</t>
-  </si>
-  <si>
     <t>ContractNumber</t>
   </si>
   <si>
-    <t>contract_number</t>
-  </si>
-  <si>
-    <t>period_of_performance_start_date</t>
-  </si>
-  <si>
     <t>DATETIME</t>
   </si>
   <si>
-    <t>period_of_performance_end_date</t>
-  </si>
-  <si>
     <t>ReportCycleID</t>
   </si>
   <si>
-    <t>report_cycle_id</t>
-  </si>
-  <si>
     <t>ReportCycleEnum</t>
   </si>
   <si>
-    <t>submission_event_number</t>
-  </si>
-  <si>
-    <t>submission_event_name</t>
-  </si>
-  <si>
-    <t>submission_event_is_wildcard</t>
-  </si>
-  <si>
     <t>BIT</t>
   </si>
   <si>
     <t>ResubmissionNumber</t>
   </si>
   <si>
-    <t>resubmission_number</t>
-  </si>
-  <si>
     <t>ReportAsOf</t>
   </si>
   <si>
-    <t>report_as_of</t>
-  </si>
-  <si>
-    <t>point_of_contact_name</t>
-  </si>
-  <si>
-    <t>point_of_contact_department</t>
-  </si>
-  <si>
-    <t>point_of_contact_telephone_number</t>
-  </si>
-  <si>
-    <t>point_of_contact_email_address</t>
-  </si>
-  <si>
     <t>DatePrepared</t>
   </si>
   <si>
-    <t>date_prepared</t>
-  </si>
-  <si>
-    <t>reporting_period_id</t>
-  </si>
-  <si>
     <t>ReportingCalendar</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>Level</t>
   </si>
   <si>
-    <t>level</t>
-  </si>
-  <si>
     <t>ParentID</t>
   </si>
   <si>
-    <t>parent_id</t>
-  </si>
-  <si>
-    <t>wbs_mapping_id</t>
-  </si>
-  <si>
     <t>ItemType</t>
   </si>
   <si>
-    <t>item_type</t>
-  </si>
-  <si>
     <t>TechnicalParameterName</t>
   </si>
   <si>
-    <t>technical_parameter_name</t>
-  </si>
-  <si>
     <t>GroupKey</t>
   </si>
   <si>
-    <t>group_key</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
-    <t>value</t>
-  </si>
-  <si>
     <t>UnitofMeasure</t>
   </si>
   <si>
-    <t>unit_of_measure</t>
-  </si>
-  <si>
     <t>UnitofMeasureQualifier</t>
   </si>
   <si>
-    <t>unit_of_measure_qualifier</t>
-  </si>
-  <si>
-    <t>estimate_or_actual</t>
-  </si>
-  <si>
     <t>Margin</t>
   </si>
   <si>
-    <t>margin</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>remarks</t>
-  </si>
-  <si>
     <t>MappingID</t>
   </si>
   <si>
-    <t>mapping_id</t>
-  </si>
-  <si>
-    <t>wbs_element_id</t>
-  </si>
-  <si>
-    <t>end_item_id</t>
-  </si>
-  <si>
-    <t>order_or_lot_id</t>
-  </si>
-  <si>
     <t>OrderOrLots</t>
   </si>
   <si>
@@ -470,6 +293,69 @@
   </si>
   <si>
     <t>LONG</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/OrganizationName</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/DivisionName</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/CAGECode</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/Location/Street</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/Location/City</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/Location/State</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/Location/ZipCode</t>
+  </si>
+  <si>
+    <t>ReportingOrganization/Location/Country</t>
+  </si>
+  <si>
+    <t>PeriodofPerformance/StartDate</t>
+  </si>
+  <si>
+    <t>PeriodofPerformance/EndDate</t>
+  </si>
+  <si>
+    <t>SubmissionEvent/Number</t>
+  </si>
+  <si>
+    <t>SubmissionEvent/Name</t>
+  </si>
+  <si>
+    <t>SubmissionEvent/IsWildcard</t>
+  </si>
+  <si>
+    <t>PointofContact/Name</t>
+  </si>
+  <si>
+    <t>PointofContact/Department</t>
+  </si>
+  <si>
+    <t>PointofContact/TelephoneNumber</t>
+  </si>
+  <si>
+    <t>PointofContact/EmailAddress</t>
+  </si>
+  <si>
+    <t>Order/LotName</t>
+  </si>
+  <si>
+    <t>Estimate/Actual</t>
+  </si>
+  <si>
+    <t>OrdersorLots</t>
+  </si>
+  <si>
+    <t>WorkBreakdownStructure</t>
   </si>
 </sst>
 </file>
@@ -513,18 +399,12 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -561,16 +441,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,33 +794,33 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>123</v>
+      <c r="A3" s="12" t="s">
+        <v>64</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>107</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3" t="b">
         <v>0</v>
@@ -948,33 +828,33 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>119</v>
+        <v>60</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>15</v>
+      <c r="C5" s="12" t="s">
+        <v>108</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" s="3" t="b">
         <v>0</v>
@@ -982,16 +862,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>120</v>
+        <v>61</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>12</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="3" t="b">
         <v>0</v>
@@ -999,16 +879,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>121</v>
+        <v>62</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="3" t="b">
         <v>0</v>
@@ -1117,7 +997,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" customWidth="1"/>
-    <col min="2" max="2" width="50" style="16" customWidth="1"/>
+    <col min="2" max="2" width="50" style="15" customWidth="1"/>
     <col min="3" max="3" width="41.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.42578125" customWidth="1"/>
     <col min="5" max="5" width="21.5703125" customWidth="1"/>
@@ -1131,43 +1011,43 @@
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>20</v>
+      <c r="B1" s="16" t="s">
+        <v>14</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>21</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F2" s="7" t="b">
         <v>0</v>
@@ -1178,16 +1058,16 @@
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>31</v>
+        <v>59</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F3" s="7" t="b">
         <v>0</v>
@@ -1198,16 +1078,16 @@
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>33</v>
+        <v>59</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F4" s="7" t="b">
         <v>0</v>
@@ -1218,25 +1098,25 @@
     </row>
     <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>34</v>
+        <v>59</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>65</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F5" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I5" s="3" t="b">
         <v>0</v>
@@ -1244,16 +1124,16 @@
     </row>
     <row r="6" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>59</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>27</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F6" s="7" t="b">
         <v>0</v>
@@ -1264,16 +1144,16 @@
     </row>
     <row r="7" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>40</v>
+        <v>59</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F7" s="7" t="b">
         <v>0</v>
@@ -1284,16 +1164,16 @@
     </row>
     <row r="8" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>41</v>
+        <v>59</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F8" s="7" t="b">
         <v>0</v>
@@ -1304,16 +1184,16 @@
     </row>
     <row r="9" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>42</v>
+        <v>59</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F9" s="7" t="b">
         <v>0</v>
@@ -1324,16 +1204,16 @@
     </row>
     <row r="10" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>43</v>
+        <v>59</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F10" s="7" t="b">
         <v>0</v>
@@ -1344,16 +1224,16 @@
     </row>
     <row r="11" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>44</v>
+        <v>59</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>69</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F11" s="7" t="b">
         <v>0</v>
@@ -1364,16 +1244,16 @@
     </row>
     <row r="12" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>45</v>
+        <v>59</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>70</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F12" s="7" t="b">
         <v>0</v>
@@ -1384,16 +1264,16 @@
     </row>
     <row r="13" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>46</v>
+        <v>59</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F13" s="7" t="b">
         <v>0</v>
@@ -1404,16 +1284,16 @@
     </row>
     <row r="14" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>47</v>
+        <v>59</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F14" s="7" t="b">
         <v>0</v>
@@ -1424,16 +1304,16 @@
     </row>
     <row r="15" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F15" s="7" t="b">
         <v>0</v>
@@ -1444,16 +1324,16 @@
     </row>
     <row r="16" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>50</v>
+        <v>59</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F16" s="7" t="b">
         <v>0</v>
@@ -1464,16 +1344,16 @@
     </row>
     <row r="17" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F17" s="7" t="b">
         <v>0</v>
@@ -1484,16 +1364,16 @@
     </row>
     <row r="18" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F18" s="7" t="b">
         <v>0</v>
@@ -1504,25 +1384,25 @@
     </row>
     <row r="19" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>32</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F19" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I19" s="3" t="b">
         <v>0</v>
@@ -1530,16 +1410,16 @@
     </row>
     <row r="20" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>59</v>
+        <v>59</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>34</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="F20" s="7" t="b">
         <v>0</v>
@@ -1550,16 +1430,16 @@
     </row>
     <row r="21" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="F21" s="7" t="b">
         <v>0</v>
@@ -1570,16 +1450,16 @@
     </row>
     <row r="22" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F22" s="7" t="b">
         <v>0</v>
@@ -1590,16 +1470,16 @@
     </row>
     <row r="23" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>74</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F23" s="7" t="b">
         <v>0</v>
@@ -1610,16 +1490,16 @@
     </row>
     <row r="24" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>67</v>
+        <v>59</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>75</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F24" s="7" t="b">
         <v>0</v>
@@ -1630,25 +1510,25 @@
     </row>
     <row r="25" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>69</v>
+        <v>59</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F25" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I25" s="3" t="b">
         <v>0</v>
@@ -1656,16 +1536,16 @@
     </row>
     <row r="26" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>71</v>
+        <v>59</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>146</v>
+        <v>87</v>
       </c>
       <c r="F26" s="7" t="b">
         <v>0</v>
@@ -1676,16 +1556,16 @@
     </row>
     <row r="27" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>72</v>
+        <v>59</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F27" s="7" t="b">
         <v>0</v>
@@ -1696,16 +1576,16 @@
     </row>
     <row r="28" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>73</v>
+        <v>59</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>78</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="F28" s="7" t="b">
         <v>0</v>
@@ -1716,16 +1596,16 @@
     </row>
     <row r="29" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>29</v>
+        <v>59</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="F29" s="7" t="b">
         <v>0</v>
@@ -1736,16 +1616,16 @@
     </row>
     <row r="30" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>78</v>
+        <v>59</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F30" s="7" t="b">
         <v>0</v>
@@ -1756,16 +1636,16 @@
     </row>
     <row r="31" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="C31" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>79</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F31" s="7" t="b">
         <v>0</v>
@@ -1776,16 +1656,16 @@
     </row>
     <row r="32" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="C32" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>80</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F32" s="7" t="b">
         <v>0</v>
@@ -1796,16 +1676,16 @@
     </row>
     <row r="33" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>81</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F33" s="7" t="b">
         <v>0</v>
@@ -1816,16 +1696,16 @@
     </row>
     <row r="34" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="C34" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>82</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F34" s="7" t="b">
         <v>0</v>
@@ -1836,16 +1716,16 @@
     </row>
     <row r="35" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>84</v>
+        <v>59</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>44</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="F35" s="7" t="b">
         <v>0</v>
@@ -1856,42 +1736,42 @@
     </row>
     <row r="36" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B36" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>29</v>
+        <v>59</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="F36" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>86</v>
+        <v>45</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I36" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>87</v>
+      <c r="A37" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F37" s="7" t="b">
         <v>1</v>
@@ -1901,17 +1781,17 @@
       </c>
     </row>
     <row r="38" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>89</v>
+      <c r="A38" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F38" s="7" t="b">
         <v>0</v>
@@ -1922,16 +1802,16 @@
     </row>
     <row r="39" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>87</v>
+        <v>60</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F39" s="7" t="b">
         <v>1</v>
@@ -1942,16 +1822,16 @@
     </row>
     <row r="40" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>89</v>
+        <v>60</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F40" s="7" t="b">
         <v>0</v>
@@ -1961,17 +1841,17 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B41" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>91</v>
+      <c r="A41" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>146</v>
+        <v>87</v>
       </c>
       <c r="F41" s="7" t="b">
         <v>0</v>
@@ -1981,43 +1861,43 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B42" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>87</v>
+      <c r="A42" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F42" s="7" t="b">
         <v>1</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I42" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B43" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>89</v>
+      <c r="A43" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F43" s="7" t="b">
         <v>0</v>
@@ -2027,26 +1907,26 @@
       </c>
     </row>
     <row r="44" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B44" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>93</v>
+      <c r="A44" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F44" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I44" s="3" t="b">
         <v>0</v>
@@ -2054,25 +1934,25 @@
     </row>
     <row r="45" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B45" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>94</v>
+        <v>61</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F45" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I45" s="3" t="b">
         <v>0</v>
@@ -2080,16 +1960,16 @@
     </row>
     <row r="46" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B46" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>96</v>
+        <v>61</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F46" s="7" t="b">
         <v>0</v>
@@ -2100,16 +1980,16 @@
     </row>
     <row r="47" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B47" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>98</v>
+        <v>61</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>50</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F47" s="7" t="b">
         <v>0</v>
@@ -2120,16 +2000,16 @@
     </row>
     <row r="48" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>100</v>
+        <v>61</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>51</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F48" s="9" t="b">
         <v>0</v>
@@ -2140,16 +2020,16 @@
     </row>
     <row r="49" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>29</v>
+        <v>61</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="F49" s="7" t="b">
         <v>0</v>
@@ -2160,16 +2040,16 @@
     </row>
     <row r="50" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B50" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>104</v>
+        <v>61</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>53</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F50" s="7" t="b">
         <v>0</v>
@@ -2180,17 +2060,17 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>106</v>
+        <v>61</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F51" s="7" t="b">
         <v>0</v>
@@ -2203,16 +2083,16 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B52" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>107</v>
+        <v>61</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F52" s="7" t="b">
         <v>0</v>
@@ -2225,16 +2105,16 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B53" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>109</v>
+        <v>61</v>
+      </c>
+      <c r="B53" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>55</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F53" s="7" t="b">
         <v>0</v>
@@ -2247,16 +2127,16 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B54" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>111</v>
+        <v>61</v>
+      </c>
+      <c r="B54" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>56</v>
       </c>
       <c r="E54" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F54" t="b">
         <v>0</v>
@@ -2267,16 +2147,16 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B55" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="C55" t="s">
-        <v>113</v>
+        <v>62</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55" s="14" t="s">
+        <v>57</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F55" s="7" t="b">
         <v>0</v>
@@ -2289,25 +2169,25 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B56" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="C56" t="s">
-        <v>114</v>
+        <v>62</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>84</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F56" s="7" t="b">
         <v>1</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I56" s="3" t="b">
         <v>0</v>
@@ -2315,26 +2195,26 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B57" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>115</v>
+        <v>62</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="11" t="s">
+        <v>9</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F57" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I57" s="3" t="b">
         <v>0</v>
@@ -2342,25 +2222,25 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B58" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>116</v>
+        <v>62</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C58" s="11" t="s">
+        <v>85</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F58" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I58" s="3" t="b">
         <v>0</v>
@@ -2368,16 +2248,16 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B59" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>111</v>
+        <v>62</v>
+      </c>
+      <c r="B59" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C59" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="E59" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F59" t="b">
         <v>0</v>
@@ -2394,27 +2274,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Notes xmlns="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="357ea1be-ddc3-494a-b1fb-24c1664aeba1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="22629126-c2bf-42e9-9255-22784a2ff070" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBC12096B4D56E43B1F5911C835D18E4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14170855f4468ba1b9b5de042169bf05">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xmlns:ns3="22629126-c2bf-42e9-9255-22784a2ff070" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="28f95ec50be93062e6854421190d2255" ns2:_="" ns3:_="">
     <xsd:import namespace="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
@@ -2669,32 +2528,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC164D1F-8249-4727-AA00-DE139E6944D4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56123D4C-31B1-40E1-921F-7AB9B3EA2A82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
-    <ds:schemaRef ds:uri="22629126-c2bf-42e9-9255-22784a2ff070"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Notes xmlns="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="357ea1be-ddc3-494a-b1fb-24c1664aeba1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="22629126-c2bf-42e9-9255-22784a2ff070" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00A6419C-415D-45D8-A760-7692730D7A3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2711,4 +2566,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC164D1F-8249-4727-AA00-DE139E6944D4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56123D4C-31B1-40E1-921F-7AB9B3EA2A82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
+    <ds:schemaRef ds:uri="22629126-c2bf-42e9-9255-22784a2ff070"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Adjusted TDR table spec to mirror FlexFile Orders/Lots structure
</commit_message>
<xml_diff>
--- a/data-raw/techdatareport-tables.xlsx
+++ b/data-raw/techdatareport-tables.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bellenbogen\Software\R\readflexfile\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C5D55F-DD37-4121-90C8-A0F24E0C5C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01870C70-A699-4288-9442-5CA52F4D169C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{B45BC891-6358-4EB6-8DF4-312547779ABA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B45BC891-6358-4EB6-8DF4-312547779ABA}"/>
   </bookViews>
   <sheets>
     <sheet name="tables" sheetId="1" r:id="rId1"/>
     <sheet name="fields" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">fields!$A$1:$I$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">fields!$A$1:$I$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="114">
   <si>
     <t>table</t>
   </si>
@@ -373,6 +373,15 @@
   </si>
   <si>
     <t>ReportingPeriodID</t>
+  </si>
+  <si>
+    <t>AppropriationTypeID</t>
+  </si>
+  <si>
+    <t>PeriodofPerformanceEndDate</t>
+  </si>
+  <si>
+    <t>PeriodofPerformanceStartDate</t>
   </si>
 </sst>
 </file>
@@ -914,7 +923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B81C7F5F-CBF8-484D-AA73-A07C6AA57BD9}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.42578125" style="6" customWidth="1"/>
@@ -1723,235 +1732,220 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A39" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>24</v>
+      <c r="A39" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="7" t="b">
+      <c r="F39" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="I39" s="6" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>44</v>
+      <c r="A40" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F40" s="7" t="b">
+      <c r="F40" s="6" t="b">
         <v>0</v>
       </c>
       <c r="I40" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>45</v>
+        <v>62</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F41" s="7" t="b">
+        <v>20</v>
+      </c>
+      <c r="F41" s="6" t="b">
         <v>0</v>
       </c>
       <c r="I41" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>24</v>
+        <v>62</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" s="7" t="b">
+        <v>33</v>
+      </c>
+      <c r="F42" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="6" t="b">
         <v>1</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I42" s="6" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>44</v>
+        <v>62</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>34</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F43" s="7" t="b">
+        <v>33</v>
+      </c>
+      <c r="F43" s="6" t="b">
         <v>0</v>
       </c>
       <c r="I43" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>46</v>
+        <v>62</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F44" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>24</v>
+        <v>36</v>
+      </c>
+      <c r="F44" s="6" t="b">
+        <v>0</v>
       </c>
       <c r="I44" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A45" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>55</v>
+      <c r="A45" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>102</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F45" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>24</v>
+        <v>36</v>
+      </c>
+      <c r="F45" s="6" t="b">
+        <v>0</v>
       </c>
       <c r="I45" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>47</v>
+      <c r="A46" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F46" s="7" t="b">
+      <c r="F46" s="6" t="b">
         <v>0</v>
       </c>
       <c r="I46" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F47" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" s="6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C48" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F48" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I48" s="12" t="b">
+      <c r="A48" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F48" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="6" t="s">
-        <v>59</v>
+      <c r="A49" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>20</v>
+        <v>45</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>68</v>
       </c>
       <c r="F49" s="7" t="b">
         <v>0</v>
@@ -1961,34 +1955,40 @@
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="6" t="s">
-        <v>59</v>
+      <c r="A50" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F50" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="I50" s="6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="6" t="s">
-        <v>59</v>
+      <c r="A51" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>20</v>
@@ -2001,20 +2001,26 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A52" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>64</v>
+      <c r="A52" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>46</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F52" s="7" t="b">
         <v>0</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="I52" s="6" t="b">
         <v>0</v>
@@ -2024,17 +2030,23 @@
       <c r="A53" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B53" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>53</v>
+      <c r="B53" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F53" s="7" t="b">
         <v>0</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="I53" s="6" t="b">
         <v>0</v>
@@ -2045,15 +2057,15 @@
         <v>59</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F54" s="6" t="b">
+      <c r="F54" s="7" t="b">
         <v>0</v>
       </c>
       <c r="I54" s="6" t="b">
@@ -2062,13 +2074,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>20</v>
@@ -2081,52 +2093,43 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A56" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F56" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I56" s="6" t="b">
+      <c r="A56" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F56" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="12" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E57" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E57" s="8" t="s">
         <v>20</v>
       </c>
       <c r="F57" s="7" t="b">
         <v>0</v>
-      </c>
-      <c r="G57" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="H57" s="6" t="s">
-        <v>24</v>
       </c>
       <c r="I57" s="6" t="b">
         <v>0</v>
@@ -2134,25 +2137,19 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>66</v>
+        <v>59</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F58" s="7" t="b">
         <v>0</v>
-      </c>
-      <c r="G58" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>24</v>
       </c>
       <c r="I58" s="6" t="b">
         <v>0</v>
@@ -2160,21 +2157,199 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F59" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F60" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B63" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F63" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F64" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I64" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F65" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I65" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F66" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I66" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B67" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C67" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E59" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="I59" s="6" t="b">
+      <c r="E67" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" s="6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2186,6 +2361,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBC12096B4D56E43B1F5911C835D18E4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14170855f4468ba1b9b5de042169bf05">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xmlns:ns3="22629126-c2bf-42e9-9255-22784a2ff070" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="28f95ec50be93062e6854421190d2255" ns2:_="" ns3:_="">
     <xsd:import namespace="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
@@ -2440,15 +2624,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2462,6 +2637,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC164D1F-8249-4727-AA00-DE139E6944D4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00A6419C-415D-45D8-A760-7692730D7A3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2476,14 +2659,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC164D1F-8249-4727-AA00-DE139E6944D4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>